<commit_message>
feat(xlsx): read hyperlinks and cell comments as read-only metadata
Hyperlinks and cell comments were preserved but invisible: a consumer could
not show a link's target or a note on a cell. `Sheet::hyperlinks()` now reads
each hyperlink's range, external target from the worksheet relationship,
in-workbook location, display text, and screen tip, and `Sheet::comments()`
reads each legacy comment's address, author, and plain text, which Excel
also writes for threaded comments.

Neither the worksheet relationships of a sheet without tables nor comments
parts were read before, so a part that does not read leaves only that
metadata out instead of failing an open that succeeded until now. A sheet
rename rewrites internal hyperlink locations as the saved part already did.

Interop, Python, Node.js, and the new `workbook_hyperlinks` and
`workbook_comments` MCP tools page through them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/binding-contract/sheet-metadata.xlsx
+++ b/binding-contract/sheet-metadata.xlsx
@@ -6,6 +6,35 @@
     <sheet name="Lists" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Ana</author>
+    <author>Bo</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+          </rPr>
+          <t>Ana:</t>
+        </r>
+        <r>
+          <t xml:space="preserve"> check &amp; confirm</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="1">
+      <text>
+        <t>Plain note</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -69,7 +98,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
     <col min="1" max="2" width="18.5" customWidth="1"/>
   </cols>
@@ -91,6 +120,10 @@
       <formula2>9</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" display="Docs" tooltip="Open the docs"/>
+    <hyperlink ref="B5:C5" location="Lists!A1" display="Lists"/>
+  </hyperlinks>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">

</xml_diff>